<commit_message>
Improve entity handling to take distinct across pairs of columns.
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/summary_control_file_w_metadata/control_file.xlsx
+++ b/inst/extdata/examples/summary_control_file_w_metadata/control_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NotBackedUp\Analytic_tool_building\IDIr\inst\extdata\examples\summary_control_file_w_metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{AF7DE648-F7AE-4A32-B583-013FB4EFF8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30B253B-65BA-4800-8C63-F8583FD43C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A516C4E9-3652-4F0D-B641-82A8595034EC}"/>
   </bookViews>
@@ -105,9 +105,6 @@
     <t>{ ifelse(edu_level &gt; 5, 1, 0) }</t>
   </si>
   <si>
-    <t>ENTITY works like DISTINCT, but with different labelling to reflect the intention.</t>
-  </si>
-  <si>
     <t>working age</t>
   </si>
   <si>
@@ -181,6 +178,9 @@
   </si>
   <si>
     <t>example_data.csv</t>
+  </si>
+  <si>
+    <t>ENTITY is similar to DISTINCT, but checks for columns with `*_min` and `*_max` suffixes and takes a distinct over the union of these columns if available. Designed for counting entities.</t>
   </si>
 </sst>
 </file>
@@ -552,102 +552,102 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="57" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -792,13 +792,13 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="F6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -806,13 +806,13 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -820,13 +820,13 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
       </c>
       <c r="F8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload of files exported from data lab
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/summary_control_file_w_metadata/control_file.xlsx
+++ b/inst/extdata/examples/summary_control_file_w_metadata/control_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NotBackedUp\Analytic_tool_building\IDIr\inst\extdata\examples\summary_control_file_w_metadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\MAA2023-46\projects\Tool development\IDIr\inst\extdata\examples\summary_control_file_w_metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30B253B-65BA-4800-8C63-F8583FD43C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEDDA88-45FB-4A0D-A61B-23E84C6A0478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A516C4E9-3652-4F0D-B641-82A8595034EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A516C4E9-3652-4F0D-B641-82A8595034EC}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="52">
   <si>
     <t>ENABLED</t>
   </si>
@@ -126,9 +126,6 @@
     <t>NOTES columns are ignored. Any other column names are ignored, but generate a warning.</t>
   </si>
   <si>
-    <t>Except for ENABLED, you can have any number of columns of each type.</t>
-  </si>
-  <si>
     <t>If the column ENABLED is included, rows set to FALSE will be omitted.</t>
   </si>
   <si>
@@ -171,9 +168,6 @@
     <t>SA</t>
   </si>
   <si>
-    <t>2025-02-10</t>
-  </si>
-  <si>
     <t>Table summarised:</t>
   </si>
   <si>
@@ -181,13 +175,31 @@
   </si>
   <si>
     <t>ENTITY is similar to DISTINCT, but checks for columns with `*_min` and `*_max` suffixes and takes a distinct over the union of these columns if available. Designed for counting entities.</t>
+  </si>
+  <si>
+    <t>Except for ENABLED and FILE, you can have any number of columns of each type.</t>
+  </si>
+  <si>
+    <t>FILE</t>
+  </si>
+  <si>
+    <t>C:/path/temp_results.csv</t>
+  </si>
+  <si>
+    <t>2025-03-04</t>
+  </si>
+  <si>
+    <t>FILE gives the file path and name where the summary output should be saved, output can be divided across multiple files.</t>
+  </si>
+  <si>
+    <t>Files and folders will be created if they do not exist and overwritten if they do exist.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,9 +239,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -248,9 +258,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -288,7 +298,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -394,7 +404,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -536,7 +546,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -544,110 +554,120 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B27B6FA9-2405-4595-95A9-CC5A985FD12F}">
-  <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:A24"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="44.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15">
+      <c r="A3" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="5" spans="1:1" ht="15">
+      <c r="A5" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="6" spans="1:1">
+      <c r="A6" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15">
+      <c r="A7" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="8" spans="1:1">
+      <c r="A8" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15">
+      <c r="A11" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="12" spans="1:1">
+      <c r="A12" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="4" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="57" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -657,8 +677,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9D0B42D-A7BA-406E-9765-3C35473088DA}">
-  <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="19.875" bestFit="1" customWidth="1"/>
@@ -669,163 +689,187 @@
     <col min="9" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
       <c r="E1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>10</v>
       </c>
       <c r="G1" t="s">
         <v>10</v>
       </c>
       <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>11</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12">
       <c r="A2" t="b">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12">
       <c r="A3" t="b">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12">
       <c r="A4" t="b">
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>14</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>15</v>
-      </c>
-      <c r="H4" t="s">
-        <v>9</v>
       </c>
       <c r="I4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" t="b">
         <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>14</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>21</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12">
       <c r="A6" t="b">
         <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
         <v>24</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12">
       <c r="A7" t="b">
         <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
         <v>22</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>7</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12">
       <c r="A8" t="b">
         <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
         <v>23</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>7</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update v0.7.1 to v0.8.3 using output from the lab
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/summary_control_file_w_metadata/control_file.xlsx
+++ b/inst/extdata/examples/summary_control_file_w_metadata/control_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\MAA2023-46\projects\Tool development\IDIr\inst\extdata\examples\summary_control_file_w_metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DCAACE-05CD-40CA-AE92-854EF73E2F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D8839AC-222D-4FBB-9154-FD5BFBCF7303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15240" xr2:uid="{A516C4E9-3652-4F0D-B641-82A8595034EC}"/>
+    <workbookView xWindow="18480" yWindow="0" windowWidth="33120" windowHeight="20400" xr2:uid="{A516C4E9-3652-4F0D-B641-82A8595034EC}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="59">
   <si>
     <t>ENABLED</t>
   </si>
@@ -198,7 +198,22 @@
     <t>SEED works like SUM but first takes modulo base 100. It is intended to support consistent random rounding.</t>
   </si>
   <si>
-    <t>2025-06-18</t>
+    <t>2025-08-22</t>
+  </si>
+  <si>
+    <t>MAX computes the maximum of non-missing values in the column.</t>
+  </si>
+  <si>
+    <t>MIN computes the maximum of non-missing values in the column.</t>
+  </si>
+  <si>
+    <t>MAX</t>
+  </si>
+  <si>
+    <t>MIN</t>
+  </si>
+  <si>
+    <t>age range</t>
   </si>
 </sst>
 </file>
@@ -560,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B27B6FA9-2405-4595-95A9-CC5A985FD12F}">
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="44.625" customWidth="1"/>
@@ -668,16 +683,26 @@
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
-      <c r="A24" s="4" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
-      <c r="A25" s="4" t="s">
+    <row r="27" spans="1:1">
+      <c r="A27" s="4" t="s">
         <v>36</v>
       </c>
     </row>
@@ -688,20 +713,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9D0B42D-A7BA-406E-9765-3C35473088DA}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="19.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="31.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="23.75" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="15" width="13.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -736,13 +754,19 @@
         <v>5</v>
       </c>
       <c r="L1" t="s">
+        <v>56</v>
+      </c>
+      <c r="M1" t="s">
+        <v>57</v>
+      </c>
+      <c r="N1" t="s">
         <v>51</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:15">
       <c r="A2" t="b">
         <v>1</v>
       </c>
@@ -762,7 +786,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:15">
       <c r="A3" t="b">
         <v>1</v>
       </c>
@@ -785,7 +809,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:15">
       <c r="A4" t="b">
         <v>1</v>
       </c>
@@ -810,11 +834,11 @@
       <c r="J4" t="s">
         <v>9</v>
       </c>
-      <c r="L4" t="s">
+      <c r="N4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:15">
       <c r="A5" t="b">
         <v>1</v>
       </c>
@@ -840,7 +864,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:15">
       <c r="A6" t="b">
         <v>1</v>
       </c>
@@ -857,7 +881,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:15">
       <c r="A7" t="b">
         <v>1</v>
       </c>
@@ -874,7 +898,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:15">
       <c r="A8" t="b">
         <v>1</v>
       </c>
@@ -889,6 +913,23 @@
       </c>
       <c r="G8" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="L9" t="s">
+        <v>6</v>
+      </c>
+      <c r="M9" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>